<commit_message>
Refresh graded props bundles and add June 9 feedback-loop reports.
Update graded enrichment and stack-70 lift analysis, regenerate mobile and UI graded prop JSON through June, and add miss attribution and void validation artifacts for 2026-06-09.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-09.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-09.xlsx
@@ -474,13 +474,13 @@
         <v>207</v>
       </c>
       <c r="E2" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F2" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G2" t="n">
-        <v>55.6</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3">
@@ -503,13 +503,13 @@
         <v>250</v>
       </c>
       <c r="E3" t="n">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F3" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G3" t="n">
-        <v>53.6</v>
+        <v>52.8</v>
       </c>
     </row>
     <row r="4">
@@ -532,13 +532,13 @@
         <v>134</v>
       </c>
       <c r="E4" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F4" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G4" t="n">
-        <v>52.2</v>
+        <v>53.7</v>
       </c>
     </row>
     <row r="5">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1035</v>
+        <v>1052</v>
       </c>
       <c r="E11" t="n">
-        <v>656</v>
+        <v>675</v>
       </c>
       <c r="F11" t="n">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="G11" t="n">
-        <v>63.4</v>
+        <v>64.2</v>
       </c>
     </row>
     <row r="12">
@@ -764,13 +764,13 @@
         <v>173</v>
       </c>
       <c r="E12" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F12" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G12" t="n">
-        <v>64.2</v>
+        <v>65.3</v>
       </c>
     </row>
     <row r="13">
@@ -822,13 +822,13 @@
         <v>303</v>
       </c>
       <c r="E14" t="n">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="F14" t="n">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="G14" t="n">
-        <v>27.1</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="15">
@@ -851,13 +851,13 @@
         <v>421</v>
       </c>
       <c r="E15" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F15" t="n">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="G15" t="n">
-        <v>17.6</v>
+        <v>17.8</v>
       </c>
     </row>
     <row r="16">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4424</v>
+        <v>4490</v>
       </c>
       <c r="E17" t="n">
-        <v>946</v>
+        <v>1004</v>
       </c>
       <c r="F17" t="n">
-        <v>3478</v>
+        <v>3486</v>
       </c>
       <c r="G17" t="n">
-        <v>21.4</v>
+        <v>22.4</v>
       </c>
     </row>
   </sheetData>
@@ -1462,13 +1462,13 @@
         <v>130</v>
       </c>
       <c r="D7" t="n">
-        <v>63.4</v>
+        <v>64.2</v>
       </c>
       <c r="E7" t="n">
-        <v>1035</v>
+        <v>1052</v>
       </c>
       <c r="F7" t="n">
-        <v>64.2</v>
+        <v>65.3</v>
       </c>
       <c r="G7" t="n">
         <v>173</v>
@@ -1480,13 +1480,13 @@
         <v>289</v>
       </c>
       <c r="J7" t="n">
-        <v>27.1</v>
+        <v>28.7</v>
       </c>
       <c r="K7" t="n">
         <v>303</v>
       </c>
       <c r="L7" t="n">
-        <v>17.6</v>
+        <v>17.8</v>
       </c>
       <c r="M7" t="n">
         <v>421</v>
@@ -1498,19 +1498,19 @@
         <v>196</v>
       </c>
       <c r="P7" t="n">
-        <v>21.4</v>
+        <v>22.4</v>
       </c>
       <c r="Q7" t="n">
-        <v>4424</v>
+        <v>4490</v>
       </c>
       <c r="R7" t="n">
-        <v>55.6</v>
+        <v>56</v>
       </c>
       <c r="S7" t="n">
         <v>207</v>
       </c>
       <c r="T7" t="n">
-        <v>52.2</v>
+        <v>53.7</v>
       </c>
       <c r="U7" t="n">
         <v>134</v>
@@ -1528,7 +1528,7 @@
         <v>304</v>
       </c>
       <c r="Z7" t="n">
-        <v>53.6</v>
+        <v>52.8</v>
       </c>
       <c r="AA7" t="n">
         <v>250</v>

</xml_diff>

<commit_message>
Daily slate 2026-06-11 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-09.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-09.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>207</v>
+        <v>235</v>
       </c>
       <c r="E2" t="n">
-        <v>116</v>
+        <v>132</v>
       </c>
       <c r="F2" t="n">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="G2" t="n">
-        <v>56</v>
+        <v>56.2</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>250</v>
+        <v>287</v>
       </c>
       <c r="E3" t="n">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="F3" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="G3" t="n">
-        <v>52.8</v>
+        <v>50.5</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E4" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F4" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G4" t="n">
-        <v>53.7</v>
+        <v>54.8</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E5" t="n">
         <v>8</v>
       </c>
       <c r="F5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G5" t="n">
-        <v>57.1</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="6">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>304</v>
+        <v>314</v>
       </c>
       <c r="E8" t="n">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F8" t="n">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="G8" t="n">
-        <v>30.3</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E9" t="n">
         <v>10</v>
       </c>
       <c r="F9" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G9" t="n">
-        <v>58.8</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>130</v>
+        <v>161</v>
       </c>
       <c r="E10" t="n">
-        <v>89</v>
+        <v>111</v>
       </c>
       <c r="F10" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="G10" t="n">
-        <v>68.5</v>
+        <v>68.90000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1052</v>
+        <v>1103</v>
       </c>
       <c r="E11" t="n">
-        <v>675</v>
+        <v>723</v>
       </c>
       <c r="F11" t="n">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="G11" t="n">
-        <v>64.2</v>
+        <v>65.5</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>173</v>
+        <v>193</v>
       </c>
       <c r="E12" t="n">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="F12" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="G12" t="n">
-        <v>65.3</v>
+        <v>66.3</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="E13" t="n">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="F13" t="n">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="G13" t="n">
-        <v>38.4</v>
+        <v>39.6</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>303</v>
+        <v>319</v>
       </c>
       <c r="E14" t="n">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="F14" t="n">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="G14" t="n">
-        <v>28.7</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>421</v>
+        <v>460</v>
       </c>
       <c r="E15" t="n">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="F15" t="n">
-        <v>346</v>
+        <v>374</v>
       </c>
       <c r="G15" t="n">
-        <v>17.8</v>
+        <v>18.7</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>196</v>
+        <v>244</v>
       </c>
       <c r="E16" t="n">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="F16" t="n">
-        <v>155</v>
+        <v>189</v>
       </c>
       <c r="G16" t="n">
-        <v>20.9</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4490</v>
+        <v>4638</v>
       </c>
       <c r="E17" t="n">
-        <v>1004</v>
+        <v>1058</v>
       </c>
       <c r="F17" t="n">
-        <v>3486</v>
+        <v>3580</v>
       </c>
       <c r="G17" t="n">
-        <v>22.4</v>
+        <v>22.8</v>
       </c>
     </row>
   </sheetData>
@@ -1106,58 +1106,58 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>90.90000000000001</v>
+        <v>79.2</v>
       </c>
       <c r="C2" t="n">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="D2" t="n">
-        <v>57.1</v>
+        <v>63.6</v>
       </c>
       <c r="E2" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F2" t="n">
-        <v>44.4</v>
+        <v>61.1</v>
       </c>
       <c r="G2" t="n">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J2" t="n">
         <v>66.7</v>
       </c>
       <c r="K2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L2" t="n">
-        <v>6.2</v>
+        <v>9.4</v>
       </c>
       <c r="M2" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="N2" t="n">
-        <v>12.5</v>
+        <v>16.7</v>
       </c>
       <c r="O2" t="n">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="P2" t="n">
-        <v>13.3</v>
+        <v>12</v>
       </c>
       <c r="Q2" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="R2" t="n">
-        <v>64.8</v>
+        <v>61.9</v>
       </c>
       <c r="S2" t="n">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="T2" t="n">
         <v>51.2</v>
@@ -1169,19 +1169,22 @@
         <v>0</v>
       </c>
       <c r="X2" t="n">
-        <v>23.7</v>
+        <v>23.3</v>
       </c>
       <c r="Y2" t="n">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="Z2" t="n">
-        <v>45</v>
+        <v>41.5</v>
       </c>
       <c r="AA2" t="n">
-        <v>40</v>
+        <v>53</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0</v>
       </c>
       <c r="AC2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE2" t="n">
         <v>0</v>
@@ -1290,32 +1293,59 @@
           <t>Avg</t>
         </is>
       </c>
+      <c r="B4" t="n">
+        <v>72.2</v>
+      </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>18</v>
+      </c>
+      <c r="D4" t="n">
+        <v>75</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="F4" t="n">
+        <v>63.6</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="H4" t="n">
+        <v>71.40000000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="J4" t="n">
+        <v>40</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="L4" t="n">
+        <v>30.4</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>23</v>
+      </c>
+      <c r="N4" t="n">
+        <v>34.5</v>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>29</v>
+      </c>
+      <c r="P4" t="n">
+        <v>26.7</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="R4" t="n">
+        <v>62.5</v>
       </c>
       <c r="S4" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="U4" t="n">
         <v>0</v>
@@ -1323,11 +1353,17 @@
       <c r="W4" t="n">
         <v>0</v>
       </c>
+      <c r="X4" t="n">
+        <v>60</v>
+      </c>
       <c r="Y4" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>58.3</v>
       </c>
       <c r="AA4" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="AC4" t="n">
         <v>0</v>
@@ -1335,8 +1371,11 @@
       <c r="AE4" t="n">
         <v>0</v>
       </c>
+      <c r="AF4" t="n">
+        <v>0</v>
+      </c>
       <c r="AG4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -1456,64 +1495,64 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>68.5</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="C7" t="n">
-        <v>130</v>
+        <v>161</v>
       </c>
       <c r="D7" t="n">
-        <v>64.2</v>
+        <v>65.5</v>
       </c>
       <c r="E7" t="n">
-        <v>1052</v>
+        <v>1103</v>
       </c>
       <c r="F7" t="n">
-        <v>65.3</v>
+        <v>66.3</v>
       </c>
       <c r="G7" t="n">
-        <v>173</v>
+        <v>193</v>
       </c>
       <c r="H7" t="n">
-        <v>38.4</v>
+        <v>39.6</v>
       </c>
       <c r="I7" t="n">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="J7" t="n">
-        <v>28.7</v>
+        <v>29.8</v>
       </c>
       <c r="K7" t="n">
-        <v>303</v>
+        <v>319</v>
       </c>
       <c r="L7" t="n">
-        <v>17.8</v>
+        <v>18.7</v>
       </c>
       <c r="M7" t="n">
-        <v>421</v>
+        <v>460</v>
       </c>
       <c r="N7" t="n">
-        <v>20.9</v>
+        <v>22.5</v>
       </c>
       <c r="O7" t="n">
-        <v>196</v>
+        <v>244</v>
       </c>
       <c r="P7" t="n">
-        <v>22.4</v>
+        <v>22.8</v>
       </c>
       <c r="Q7" t="n">
-        <v>4490</v>
+        <v>4638</v>
       </c>
       <c r="R7" t="n">
-        <v>56</v>
+        <v>56.2</v>
       </c>
       <c r="S7" t="n">
-        <v>207</v>
+        <v>235</v>
       </c>
       <c r="T7" t="n">
-        <v>53.7</v>
+        <v>54.8</v>
       </c>
       <c r="U7" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="V7" t="n">
         <v>33.3</v>
@@ -1522,22 +1561,22 @@
         <v>3</v>
       </c>
       <c r="X7" t="n">
-        <v>30.3</v>
+        <v>30.6</v>
       </c>
       <c r="Y7" t="n">
-        <v>304</v>
+        <v>314</v>
       </c>
       <c r="Z7" t="n">
-        <v>52.8</v>
+        <v>50.5</v>
       </c>
       <c r="AA7" t="n">
-        <v>250</v>
+        <v>287</v>
       </c>
       <c r="AB7" t="n">
-        <v>57.1</v>
+        <v>53.3</v>
       </c>
       <c r="AC7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="AD7" t="n">
         <v>66.7</v>
@@ -1546,10 +1585,10 @@
         <v>3</v>
       </c>
       <c r="AF7" t="n">
-        <v>58.8</v>
+        <v>50</v>
       </c>
       <c r="AG7" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>